<commit_message>
Mark tropical sage non-native and record checks under Aydin
The USF Atlas lists Salvia coccinea as Not Native, so it leaves the
natives and recommended lists and goes on a new Atlas non-natives list
that is checked before USDA. checked_by now reads Aydin. Adds the
approved plan for EcoScan plant cards, choose by name, and site filters.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plant-checklist.xlsx
+++ b/docs/plant-checklist.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1807,12 +1807,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Tropical sage</t>
+          <t>Fakahatchee grass</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Salvia coccinea</t>
+          <t>Tripsacum dactyloides</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Hummingbirds and butterflies drink from its red flowers, and other birds eat its seeds.</t>
+          <t>Caterpillars of two kinds of skipper butterflies eat its leaves, and birds find seeds and insects in it.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Full sun to light shade; 2 to 4 feet tall.</t>
+          <t>Full sun to light shade; 3 to 4 feet tall, up to 6 feet when blooming.</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -1846,7 +1846,7 @@
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>lantana (Lantana strigocamara)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr"/>
@@ -1861,12 +1861,12 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Fakahatchee grass</t>
+          <t>Muhly grass</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Tripsacum dactyloides</t>
+          <t>Muhlenbergia capillaris</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Caterpillars of two kinds of skipper butterflies eat its leaves, and birds find seeds and insects in it.</t>
+          <t>Its thick clumps give small animals a good place to hide.</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Full sun to light shade; 3 to 4 feet tall, up to 6 feet when blooming.</t>
+          <t>Full sun to light shade; 2 to 3 feet tall, up to 5 feet when blooming.</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1915,12 +1915,12 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Muhly grass</t>
+          <t>Saw palmetto</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Muhlenbergia capillaris</t>
+          <t>Serenoa repens</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Its thick clumps give small animals a good place to hide.</t>
+          <t>Caterpillars of the palmetto skipper and monk skipper butterflies eat its leaves, and deer, bears and turkeys eat its fruit.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Full sun to light shade; 2 to 3 feet tall, up to 5 feet when blooming.</t>
+          <t>Full sun to light shade; 4 to 6 feet tall, usually wider than tall.</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -1948,8 +1948,16 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>It grows very slowly, so start with the biggest plant you can.</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
       <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr"/>
       <c r="M24" s="4" t="inlineStr">
@@ -1969,12 +1977,12 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Saw palmetto</t>
+          <t>Black-eyed Susan</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Serenoa repens</t>
+          <t>Rudbeckia hirta</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -1984,7 +1992,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Caterpillars of the palmetto skipper and monk skipper butterflies eat its leaves, and deer, bears and turkeys eat its fruit.</t>
+          <t>Native bees and other helpful insects visit its flowers, and birds eat its seeds.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1994,7 +2002,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Full sun to light shade; 4 to 6 feet tall, usually wider than tall.</t>
+          <t>Full sun; 1 to 3 feet tall.</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -2002,16 +2010,8 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>It grows very slowly, so start with the biggest plant you can.</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr"/>
       <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="4" t="inlineStr"/>
       <c r="M25" s="4" t="inlineStr">
@@ -2031,12 +2031,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Black-eyed Susan</t>
+          <t>Wand goldenrod</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Rudbeckia hirta</t>
+          <t>Solidago stricta</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Native bees and other helpful insects visit its flowers, and birds eat its seeds.</t>
+          <t>Native bees visit its flowers, and birds find lots of insects on it to eat.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Full sun; 1 to 3 feet tall.</t>
+          <t>Full sun; under a foot tall, up to 4 feet when blooming.</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Wand goldenrod</t>
+          <t>Coastal Plain willow</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Solidago stricta</t>
+          <t>Salix caroliniana</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Native bees visit its flowers, and birds find lots of insects on it to eat.</t>
+          <t>It is the only native plant whose leaves viceroy butterfly caterpillars eat, and io moth caterpillars eat it too.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Full sun; under a foot tall, up to 4 feet when blooming.</t>
+          <t>Full sun to light shade; 15 to 30 feet tall in South Florida.</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2118,13 +2118,21 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr"/>
-      <c r="J27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>It needs moist or wet soil and won't handle long dry spells.</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
       <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>punktree (Melaleuca quinquenervia)</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr"/>
@@ -2139,12 +2147,12 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Coastal Plain willow</t>
+          <t>Wild lime</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Salix caroliniana</t>
+          <t>Zanthoxylum fagara</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2154,7 +2162,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>It is the only native plant whose leaves viceroy butterfly caterpillars eat, and io moth caterpillars eat it too.</t>
+          <t>Caterpillars of the giant swallowtail butterfly eat its leaves.</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2164,7 +2172,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Full sun to light shade; 15 to 30 feet tall in South Florida.</t>
+          <t>Full sun; 10 to 20 feet tall, about as wide.</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2174,7 +2182,7 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>It needs moist or wet soil and won't handle long dry spells.</t>
+          <t>Its branches have sharp, hooked thorns, so keep it away from paths.</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2186,7 +2194,7 @@
       <c r="L28" s="4" t="inlineStr"/>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>punktree (Melaleuca quinquenervia)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr"/>
@@ -2201,12 +2209,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Wild lime</t>
+          <t>Swamp milkweed</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Zanthoxylum fagara</t>
+          <t>Asclepias incarnata</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -2216,7 +2224,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Caterpillars of the giant swallowtail butterfly eat its leaves.</t>
+          <t>Caterpillars of the monarch and queen butterflies eat its leaves, and hummingbirds, bees and butterflies drink from its flowers.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2226,7 +2234,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Full sun; 10 to 20 feet tall, about as wide.</t>
+          <t>Light to moderate shade, or full sun; 3 to 5 feet tall.</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2236,7 +2244,7 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Its branches have sharp, hooked thorns, so keep it away from paths.</t>
+          <t>It needs moist or wet soil and won't handle long dry spells.</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -2263,12 +2271,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Swamp milkweed</t>
+          <t>Inkberry</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Asclepias incarnata</t>
+          <t>Scaevola plumieri</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -2278,7 +2286,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Caterpillars of the monarch and queen butterflies eat its leaves, and hummingbirds, bees and butterflies drink from its flowers.</t>
+          <t>Its black berries and low branches give food and cover to wildlife near the beach.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -2288,7 +2296,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Light to moderate shade, or full sun; 3 to 5 feet tall.</t>
+          <t>Full sun; 2 to 5 feet tall, usually wider than tall.</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -2296,21 +2304,13 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>It needs moist or wet soil and won't handle long dry spells.</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr"/>
       <c r="K30" s="4" t="inlineStr"/>
       <c r="L30" s="4" t="inlineStr"/>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>beach naupaka (Scaevola taccada)</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr"/>
@@ -2325,12 +2325,12 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Inkberry</t>
+          <t>Wild sage</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Scaevola plumieri</t>
+          <t>Lantana involucrata</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Its black berries and low branches give food and cover to wildlife near the beach.</t>
+          <t>Dozens of kinds of butterflies drink from its flowers, and many birds eat its purple fruit.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Full sun; 2 to 5 feet tall, usually wider than tall.</t>
+          <t>Full sun; 4 to 8 feet tall, about as wide.</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -2358,13 +2358,21 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Plain lantana (Lantana strigocamara) is invasive, so make sure the tag says Lantana involucrata.</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr"/>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>beach naupaka (Scaevola taccada)</t>
+          <t>lantana (Lantana strigocamara)</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr"/>
@@ -2373,71 +2381,9 @@
       <c r="Q31" s="4" t="inlineStr"/>
       <c r="R31" s="4" t="inlineStr"/>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Wild sage</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Lantana involucrata</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Open page</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Dozens of kinds of butterflies drink from its flowers, and many birds eat its purple fruit.</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Full sun; 4 to 8 feet tall, about as wide.</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>Plain lantana (Lantana strigocamara) is invasive, so make sure the tag says Lantana involucrata.</t>
-        </is>
-      </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr"/>
-      <c r="L32" s="4" t="inlineStr"/>
-      <c r="M32" s="4" t="inlineStr">
-        <is>
-          <t>lantana (Lantana strigocamara)</t>
-        </is>
-      </c>
-      <c r="N32" s="4" t="inlineStr"/>
-      <c r="O32" s="4" t="inlineStr"/>
-      <c r="P32" s="4" t="inlineStr"/>
-      <c r="Q32" s="4" t="inlineStr"/>
-      <c r="R32" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="N2:Q32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:Q31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2522,35 +2468,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId106"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>